<commit_message>
Update survey results for REMIND
</commit_message>
<xml_diff>
--- a/data/survey/storage-in-IAMs_survey.xlsx
+++ b/data/survey/storage-in-IAMs_survey.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zakeri\My Drive\Job\IIASA\Projects\ECEMF\WP1\Storage survey\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zakeri\My Drive\Job\IIASA\Projects\ECEMF\WP1\Storage survey\storage-iam-paper\data\survey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CA34654-4CFB-4F1E-A4EA-9B763D59984A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B097E63-4CA6-4CFF-A3A3-5564705889EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -5932,7 +5932,7 @@
         <v>1</v>
       </c>
       <c r="J4">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -5976,7 +5976,7 @@
         <v>424</v>
       </c>
       <c r="J5" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="K5" t="s">
         <v>288</v>
@@ -6386,7 +6386,7 @@
         <v>1</v>
       </c>
       <c r="J18">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="K18">
         <v>0</v>
@@ -6718,7 +6718,7 @@
         <v>424</v>
       </c>
       <c r="J26" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="K26" t="s">
         <v>288</v>
@@ -6759,7 +6759,7 @@
         <v>424</v>
       </c>
       <c r="J27" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="K27" t="s">
         <v>288</v>
@@ -8582,7 +8582,7 @@
         <v>1.25</v>
       </c>
       <c r="J78">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="K78">
         <v>0</v>
@@ -8708,7 +8708,7 @@
         <v>424</v>
       </c>
       <c r="J81" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="K81" t="s">
         <v>288</v>
@@ -8790,7 +8790,7 @@
         <v>424</v>
       </c>
       <c r="J83" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="K83" t="s">
         <v>288</v>
@@ -8954,7 +8954,7 @@
         <v>424</v>
       </c>
       <c r="J87" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="K87" t="s">
         <v>288</v>
@@ -9332,7 +9332,7 @@
       </c>
       <c r="J99" s="7">
         <f t="shared" si="0"/>
-        <v>5.5</v>
+        <v>7.25</v>
       </c>
       <c r="K99" s="7">
         <v>0</v>
@@ -10119,7 +10119,7 @@
         <v>0.75</v>
       </c>
       <c r="J121">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="K121">
         <v>0.25</v>
@@ -10409,7 +10409,7 @@
         <v>425</v>
       </c>
       <c r="J128" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="K128" t="s">
         <v>425</v>
@@ -10491,7 +10491,7 @@
         <v>0.5</v>
       </c>
       <c r="J131">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="K131">
         <v>0.75</v>
@@ -10755,7 +10755,7 @@
         <v>425</v>
       </c>
       <c r="J137" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="K137" t="s">
         <v>424</v>
@@ -10799,7 +10799,7 @@
         <v>0.5</v>
       </c>
       <c r="J139">
-        <v>0.75</v>
+        <v>1.5</v>
       </c>
       <c r="K139">
         <v>1.5</v>
@@ -11048,7 +11048,7 @@
         <v>425</v>
       </c>
       <c r="J145" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="K145" t="s">
         <v>424</v>
@@ -11171,7 +11171,7 @@
         <v>425</v>
       </c>
       <c r="J148" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="K148" t="s">
         <v>425</v>
@@ -11253,7 +11253,7 @@
         <v>425</v>
       </c>
       <c r="J150" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="K150" t="s">
         <v>424</v>
@@ -11420,7 +11420,7 @@
       </c>
       <c r="J155" s="7">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>6.25</v>
       </c>
       <c r="K155" s="7">
         <f t="shared" si="1"/>
@@ -11461,7 +11461,7 @@
         <v>0</v>
       </c>
       <c r="J158">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K158">
         <v>1</v>
@@ -11583,7 +11583,7 @@
       </c>
       <c r="J161" s="7">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K161" s="7">
         <f t="shared" si="2"/>
@@ -11803,28 +11803,28 @@
         <v>Storage technology</v>
       </c>
       <c r="E170">
-        <f>E2+E4+E8+E16</f>
+        <f t="shared" ref="E170:J170" si="4">E2+E4+E8+E16</f>
         <v>3</v>
       </c>
       <c r="F170">
-        <f>F2+F4+F8+F16</f>
+        <f t="shared" si="4"/>
         <v>2.25</v>
       </c>
       <c r="G170">
-        <f>G2+G4+G8+G16</f>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="H170">
-        <f>H2+H4+H8+H16</f>
+        <f t="shared" si="4"/>
         <v>2.75</v>
       </c>
       <c r="I170">
-        <f>I2+I4+I8+I16</f>
+        <f t="shared" si="4"/>
         <v>2.75</v>
       </c>
       <c r="J170">
-        <f>J2+J4+J8+J16</f>
-        <v>2</v>
+        <f t="shared" si="4"/>
+        <v>2.5</v>
       </c>
       <c r="K170">
         <v>0</v>
@@ -11848,34 +11848,34 @@
         <v>1.75</v>
       </c>
       <c r="F171">
-        <f t="shared" ref="F171:M171" si="4">F18+F34</f>
+        <f t="shared" ref="F171:M171" si="5">F18+F34</f>
         <v>1.75</v>
       </c>
       <c r="G171">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="H171">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1.75</v>
       </c>
       <c r="I171">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="J171">
-        <f t="shared" si="4"/>
-        <v>1.5</v>
+        <f t="shared" si="5"/>
+        <v>2</v>
       </c>
       <c r="K171">
         <v>0</v>
       </c>
       <c r="L171">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="M171" s="14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>5</v>
       </c>
     </row>
@@ -11885,39 +11885,39 @@
         <v>319</v>
       </c>
       <c r="E172">
-        <f>E42+E49+E56+E62+E71</f>
+        <f t="shared" ref="E172:M172" si="6">E42+E49+E56+E62+E71</f>
         <v>2.75</v>
       </c>
       <c r="F172">
-        <f>F42+F49+F56+F62+F71</f>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="G172">
-        <f>G42+G49+G56+G62+G71</f>
+        <f t="shared" si="6"/>
         <v>1.5</v>
       </c>
       <c r="H172">
-        <f>H42+H49+H56+H62+H71</f>
+        <f t="shared" si="6"/>
         <v>3.25</v>
       </c>
       <c r="I172">
-        <f>I42+I49+I56+I62+I71</f>
+        <f t="shared" si="6"/>
         <v>1.5</v>
       </c>
       <c r="J172">
-        <f>J42+J49+J56+J62+J71</f>
+        <f t="shared" si="6"/>
         <v>0.75</v>
       </c>
       <c r="K172">
-        <f>K42+K49+K56+K62+K71</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="L172">
-        <f>L42+L49+L56+L62+L71</f>
+        <f t="shared" si="6"/>
         <v>1.25</v>
       </c>
       <c r="M172" s="14">
-        <f>M42+M49+M56+M62+M71</f>
+        <f t="shared" si="6"/>
         <v>5.25</v>
       </c>
     </row>
@@ -11927,39 +11927,39 @@
         <v>562</v>
       </c>
       <c r="E173">
-        <f>E78+E89+E96</f>
+        <f t="shared" ref="E173:M173" si="7">E78+E89+E96</f>
         <v>2.25</v>
       </c>
       <c r="F173">
-        <f>F78+F89+F96</f>
+        <f t="shared" si="7"/>
         <v>1.25</v>
       </c>
       <c r="G173">
-        <f>G78+G89+G96</f>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="H173">
-        <f>H78+H89+H96</f>
+        <f t="shared" si="7"/>
         <v>2.25</v>
       </c>
       <c r="I173">
-        <f>I78+I89+I96</f>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="J173">
-        <f>J78+J89+J96</f>
-        <v>1.25</v>
+        <f t="shared" si="7"/>
+        <v>2</v>
       </c>
       <c r="K173">
-        <f>K78+K89+K96</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="L173">
-        <f>L78+L89+L96</f>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="M173" s="14">
-        <f>M78+M89+M96</f>
+        <f t="shared" si="7"/>
         <v>4</v>
       </c>
     </row>
@@ -11979,35 +11979,35 @@
         <v>1.25</v>
       </c>
       <c r="F175">
-        <f t="shared" ref="F175:M175" si="5">F101</f>
+        <f t="shared" ref="F175:M175" si="8">F101</f>
         <v>1</v>
       </c>
       <c r="G175">
-        <f t="shared" si="5"/>
+        <f t="shared" si="8"/>
         <v>1.75</v>
       </c>
       <c r="H175">
-        <f t="shared" si="5"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="I175">
-        <f t="shared" si="5"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="J175">
-        <f t="shared" si="5"/>
+        <f t="shared" si="8"/>
         <v>1.25</v>
       </c>
       <c r="K175">
-        <f t="shared" si="5"/>
+        <f t="shared" si="8"/>
         <v>1.25</v>
       </c>
       <c r="L175">
-        <f t="shared" si="5"/>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="M175" s="14">
-        <f t="shared" si="5"/>
+        <f t="shared" si="8"/>
         <v>1.75</v>
       </c>
     </row>
@@ -12021,35 +12021,35 @@
         <v>1.5</v>
       </c>
       <c r="F176">
-        <f t="shared" ref="F176:M176" si="6">F111</f>
+        <f t="shared" ref="F176:M176" si="9">F111</f>
         <v>1</v>
       </c>
       <c r="G176">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>1.75</v>
       </c>
       <c r="H176">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>1.5</v>
       </c>
       <c r="I176">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>1.25</v>
       </c>
       <c r="J176">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>1.25</v>
       </c>
       <c r="K176">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>1.25</v>
       </c>
       <c r="L176">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>1.25</v>
       </c>
       <c r="M176" s="14">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>2</v>
       </c>
     </row>
@@ -12063,35 +12063,35 @@
         <v>1.25</v>
       </c>
       <c r="F177">
-        <f t="shared" ref="F177:M177" si="7">F121+F131</f>
+        <f t="shared" ref="F177:M177" si="10">F121+F131</f>
         <v>1.5</v>
       </c>
       <c r="G177">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>1.75</v>
       </c>
       <c r="H177">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>2.5</v>
       </c>
       <c r="I177">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>1.25</v>
       </c>
       <c r="J177">
-        <f t="shared" si="7"/>
-        <v>1.75</v>
+        <f t="shared" si="10"/>
+        <v>2.25</v>
       </c>
       <c r="K177">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="L177">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.5</v>
       </c>
       <c r="M177" s="14">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3.25</v>
       </c>
     </row>
@@ -12105,35 +12105,35 @@
         <v>1.5</v>
       </c>
       <c r="F178">
-        <f t="shared" ref="F178:M178" si="8">F139</f>
+        <f t="shared" ref="F178:M178" si="11">F139</f>
         <v>0.5</v>
       </c>
       <c r="G178">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>1.5</v>
       </c>
       <c r="H178">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>1.75</v>
       </c>
       <c r="I178">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0.5</v>
       </c>
       <c r="J178">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
+        <v>1.5</v>
+      </c>
+      <c r="K178">
+        <f t="shared" si="11"/>
+        <v>1.5</v>
+      </c>
+      <c r="L178">
+        <f t="shared" si="11"/>
         <v>0.75</v>
       </c>
-      <c r="K178">
-        <f t="shared" si="8"/>
-        <v>1.5</v>
-      </c>
-      <c r="L178">
-        <f t="shared" si="8"/>
-        <v>0.75</v>
-      </c>
       <c r="M178" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>3.5</v>
       </c>
     </row>
@@ -12153,35 +12153,35 @@
         <v>2</v>
       </c>
       <c r="F180">
-        <f t="shared" ref="F180:M180" si="9">F158</f>
+        <f t="shared" ref="F180:M180" si="12">F158</f>
         <v>0</v>
       </c>
       <c r="G180">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>3</v>
       </c>
       <c r="H180">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="I180">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="J180">
-        <f t="shared" si="9"/>
-        <v>1</v>
+        <f t="shared" si="12"/>
+        <v>0</v>
       </c>
       <c r="K180">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="L180">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="M180" s="14">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>4</v>
       </c>
     </row>
@@ -12198,7 +12198,7 @@
         <v>0</v>
       </c>
       <c r="G181">
-        <f t="shared" ref="G181:M181" si="10">G159+G160</f>
+        <f t="shared" ref="G181:M181" si="13">G159+G160</f>
         <v>1</v>
       </c>
       <c r="H181">
@@ -12208,18 +12208,18 @@
         <v>0</v>
       </c>
       <c r="J181">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="K181">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="L181">
         <v>0</v>
       </c>
       <c r="M181" s="14">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>2</v>
       </c>
     </row>
@@ -12239,35 +12239,35 @@
         <v>1</v>
       </c>
       <c r="F183">
-        <f t="shared" ref="F183:M183" si="11">F164</f>
+        <f t="shared" ref="F183:M183" si="14">F164</f>
         <v>1</v>
       </c>
       <c r="G183">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="H183">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="I183">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="J183">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>2</v>
       </c>
       <c r="K183">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>1</v>
       </c>
       <c r="L183">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="M183" s="14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>4</v>
       </c>
     </row>
@@ -12283,35 +12283,35 @@
         <v>0</v>
       </c>
       <c r="F184" s="16">
-        <f t="shared" ref="F184:M184" si="12">F165+F166</f>
+        <f t="shared" ref="F184:M184" si="15">F165+F166</f>
         <v>0</v>
       </c>
       <c r="G184" s="16">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0.5</v>
       </c>
       <c r="H184" s="16">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0.5</v>
       </c>
       <c r="I184" s="16">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="J184" s="16">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0.5</v>
       </c>
       <c r="K184" s="16">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0.5</v>
       </c>
       <c r="L184" s="16">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="M184" s="17">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>4</v>
       </c>
     </row>
@@ -12386,7 +12386,7 @@
       </c>
       <c r="G2">
         <f>'SRF-detailed'!J99</f>
-        <v>5.5</v>
+        <v>7.25</v>
       </c>
       <c r="H2">
         <f>'SRF-detailed'!K99</f>
@@ -12427,7 +12427,7 @@
       </c>
       <c r="G3">
         <f>'SRF-detailed'!J155</f>
-        <v>5</v>
+        <v>6.25</v>
       </c>
       <c r="H3">
         <f>'SRF-detailed'!K155</f>
@@ -12468,7 +12468,7 @@
       </c>
       <c r="G4">
         <f>'SRF-detailed'!J161</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H4">
         <f>'SRF-detailed'!K161</f>
@@ -12638,7 +12638,7 @@
         <v>1</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3">
         <v>0</v>
@@ -12648,7 +12648,7 @@
       </c>
       <c r="K3">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
@@ -13201,7 +13201,7 @@
       </c>
       <c r="H2">
         <f>'SRF-detailed'!J170</f>
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="I2">
         <f>'SRF-detailed'!K170</f>
@@ -13245,7 +13245,7 @@
       </c>
       <c r="H3">
         <f>'SRF-detailed'!J171</f>
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="I3">
         <f>'SRF-detailed'!K171</f>
@@ -13333,7 +13333,7 @@
       </c>
       <c r="H5">
         <f>'SRF-detailed'!J173</f>
-        <v>1.25</v>
+        <v>2</v>
       </c>
       <c r="I5">
         <f>'SRF-detailed'!K173</f>
@@ -13377,7 +13377,7 @@
       </c>
       <c r="H6">
         <f t="shared" si="0"/>
-        <v>5.5</v>
+        <v>7.25</v>
       </c>
       <c r="I6">
         <f t="shared" si="0"/>
@@ -13509,7 +13509,7 @@
       </c>
       <c r="H9">
         <f>'SRF-detailed'!J177</f>
-        <v>1.75</v>
+        <v>2.25</v>
       </c>
       <c r="I9">
         <f>'SRF-detailed'!K177</f>
@@ -13553,7 +13553,7 @@
       </c>
       <c r="H10">
         <f>'SRF-detailed'!J178</f>
-        <v>0.75</v>
+        <v>1.5</v>
       </c>
       <c r="I10">
         <f>'SRF-detailed'!K178</f>
@@ -13597,7 +13597,7 @@
       </c>
       <c r="H11">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>6.25</v>
       </c>
       <c r="I11">
         <f t="shared" si="1"/>
@@ -13641,7 +13641,7 @@
       </c>
       <c r="H12">
         <f>'SRF-detailed'!J180</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I12">
         <f>'SRF-detailed'!K180</f>
@@ -13729,7 +13729,7 @@
       </c>
       <c r="H14">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I14">
         <f t="shared" si="2"/>

</xml_diff>